<commit_message>
fix(demo): supprime les Centre de coût dupliqués dans l'arborescence financière
Les 6 lignes "Centre de coût" d'origine pointaient encore directement vers
le P&L (niveau grand-parent) au lieu de la nouvelle Catégorie intermédiaire,
et faisaient doublon avec les lignes équivalentes ajoutées pour le passage
à 4 étages. Cela provoquait une erreur d'import ("Code parent introuvable
dans le niveau Catégorie").

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/arborescence_financiere_demo.xlsx
+++ b/demo/arborescence_financiere_demo.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D66"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,132 +541,132 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CC-PROC-001</t>
+          <t>CAT-REV-PROD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Achats directs</t>
+          <t>Ventes Produits</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>REV</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CC-OPS-001</t>
+          <t>CAT-REV-SERV</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Prestations &amp; Services</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>REV</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CC-SGA-001</t>
+          <t>CAT-COGS-ACH</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Achats &amp; Approvisionnement</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SGA</t>
+          <t>COGS</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CC-SGA-002</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ventes</t>
+          <t>Production &amp; Industriel</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SGA</t>
+          <t>COGS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CC-GA-001</t>
+          <t>CAT-COGS-LOG</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Supply Chain &amp; Logistique</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>COGS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CC-GA-002</t>
+          <t>CAT-SGA-MKT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>SGA</t>
         </is>
       </c>
     </row>
@@ -678,17 +678,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAT-REV-PROD</t>
+          <t>CAT-SGA-VTE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ventes Produits</t>
+          <t>Ventes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>REV</t>
+          <t>SGA</t>
         </is>
       </c>
     </row>
@@ -700,17 +700,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CAT-REV-SERV</t>
+          <t>CAT-GA-SUP</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Prestations &amp; Services</t>
+          <t>Fonctions support</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>REV</t>
+          <t>GA</t>
         </is>
       </c>
     </row>
@@ -722,17 +722,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CAT-COGS-ACH</t>
+          <t>CAT-GA-IT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Achats &amp; Approvisionnement</t>
+          <t>IT &amp; Digital</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>GA</t>
         </is>
       </c>
     </row>
@@ -744,149 +744,149 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-GA-QUAL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Production &amp; Industriel</t>
+          <t>Qualité &amp; Conformité</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>GA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CAT-COGS-LOG</t>
+          <t>CC-PROC-001</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Supply Chain &amp; Logistique</t>
+          <t>Achats directs</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>CAT-COGS-ACH</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CAT-SGA-MKT</t>
+          <t>CC-PROC-002</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Achats indirects &amp; emballages</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SGA</t>
+          <t>CAT-COGS-ACH</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CAT-SGA-VTE</t>
+          <t>CC-OPS-001</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ventes</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>SGA</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CAT-GA-SUP</t>
+          <t>CC-PROD-001</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fonctions support</t>
+          <t>Production – Usine de Vitré</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAT-GA-IT</t>
+          <t>CC-PROD-002</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>IT &amp; Digital</t>
+          <t>Production – Usine de Hambourg</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAT-GA-QUAL</t>
+          <t>CC-PROD-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Qualité &amp; Conformité</t>
+          <t>Production – Usine de Valence</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
@@ -898,17 +898,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CC-PROC-001</t>
+          <t>CC-PROD-004</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Achats directs</t>
+          <t>Production – Usine de Green Bay</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CAT-COGS-ACH</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CC-PROC-002</t>
+          <t>CC-MAINT-001</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Achats indirects &amp; emballages</t>
+          <t>Maintenance industrielle</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CAT-COGS-ACH</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
@@ -942,12 +942,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CC-OPS-001</t>
+          <t>CC-ENER-001</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Énergie &amp; Utilités</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -964,17 +964,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CC-PROD-001</t>
+          <t>CC-LOG-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Production – Usine de Vitré</t>
+          <t>Logistique inter-usines</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-COGS-LOG</t>
         </is>
       </c>
     </row>
@@ -986,17 +986,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CC-PROD-002</t>
+          <t>CC-SGA-001</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Production – Usine de Hambourg</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-SGA-MKT</t>
         </is>
       </c>
     </row>
@@ -1008,17 +1008,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CC-PROD-003</t>
+          <t>CC-SGA-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Production – Usine de Valence</t>
+          <t>Ventes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-SGA-VTE</t>
         </is>
       </c>
     </row>
@@ -1030,17 +1030,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CC-PROD-004</t>
+          <t>CC-GA-001</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Production – Usine de Green Bay</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-GA-IT</t>
         </is>
       </c>
     </row>
@@ -1052,17 +1052,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CC-MAINT-001</t>
+          <t>CC-GA-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Maintenance industrielle</t>
+          <t>RH</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-GA-SUP</t>
         </is>
       </c>
     </row>
@@ -1074,149 +1074,149 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CC-ENER-001</t>
+          <t>CC-QUAL-001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Énergie &amp; Utilités</t>
+          <t>Qualité</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-GA-QUAL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CC-LOG-002</t>
+          <t>CC-PROC-001-PD1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Logistique inter-usines</t>
+          <t>Matières premières</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CAT-COGS-LOG</t>
+          <t>CC-PROC-001</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CC-SGA-001</t>
+          <t>CC-PROC-001-PD2</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Emballages</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>CAT-SGA-MKT</t>
+          <t>CC-PROC-001</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CC-SGA-002</t>
+          <t>CC-PROC-002-PD1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ventes</t>
+          <t>Emballages plastiques</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CAT-SGA-VTE</t>
+          <t>CC-PROC-002</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CC-GA-001</t>
+          <t>CC-PROC-002-PD2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fournitures indirectes</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CAT-GA-IT</t>
+          <t>CC-PROC-002</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CC-GA-002</t>
+          <t>CC-OPS-001-PD1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>Main d'œuvre directe</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>CAT-GA-SUP</t>
+          <t>CC-OPS-001</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CC-QUAL-001</t>
+          <t>CC-OPS-001-PD2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Qualité</t>
+          <t>Consommables production</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CAT-GA-QUAL</t>
+          <t>CC-OPS-001</t>
         </is>
       </c>
     </row>
@@ -1228,17 +1228,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CC-PROC-001-PD1</t>
+          <t>CC-PROD-001-PD1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Matières premières</t>
+          <t>Main d'œuvre directe</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CC-PROC-001</t>
+          <t>CC-PROD-001</t>
         </is>
       </c>
     </row>
@@ -1250,17 +1250,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CC-PROC-001-PD2</t>
+          <t>CC-PROD-001-PD2</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Emballages</t>
+          <t>Énergie ligne UHT</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CC-PROC-001</t>
+          <t>CC-PROD-001</t>
         </is>
       </c>
     </row>
@@ -1272,17 +1272,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CC-PROC-002-PD1</t>
+          <t>CC-PROD-002-PD1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Emballages plastiques</t>
+          <t>Main d'œuvre directe</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>CC-PROC-002</t>
+          <t>CC-PROD-002</t>
         </is>
       </c>
     </row>
@@ -1294,17 +1294,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CC-PROC-002-PD2</t>
+          <t>CC-PROD-002-PD2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Fournitures indirectes</t>
+          <t>Matière première laitière</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CC-PROC-002</t>
+          <t>CC-PROD-002</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CC-OPS-001-PD1</t>
+          <t>CC-PROD-003-PD1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CC-OPS-001</t>
+          <t>CC-PROD-003</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CC-OPS-001-PD2</t>
+          <t>CC-PROD-003-PD2</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Consommables production</t>
+          <t>Consommables conditionnement</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>CC-OPS-001</t>
+          <t>CC-PROD-003</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CC-PROD-001-PD1</t>
+          <t>CC-PROD-004-PD1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>CC-PROD-001</t>
+          <t>CC-PROD-004</t>
         </is>
       </c>
     </row>
@@ -1382,17 +1382,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CC-PROD-001-PD2</t>
+          <t>CC-PROD-004-PD2</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Énergie ligne UHT</t>
+          <t>Consommables conditionnement</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>CC-PROD-001</t>
+          <t>CC-PROD-004</t>
         </is>
       </c>
     </row>
@@ -1404,17 +1404,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CC-PROD-002-PD1</t>
+          <t>CC-MAINT-001-PD1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Main d'œuvre directe</t>
+          <t>Pièces détachées</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>CC-PROD-002</t>
+          <t>CC-MAINT-001</t>
         </is>
       </c>
     </row>
@@ -1426,17 +1426,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CC-PROD-002-PD2</t>
+          <t>CC-MAINT-001-PD2</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Matière première laitière</t>
+          <t>Contrats de maintenance</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>CC-PROD-002</t>
+          <t>CC-MAINT-001</t>
         </is>
       </c>
     </row>
@@ -1448,17 +1448,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CC-PROD-003-PD1</t>
+          <t>CC-ENER-001-PD1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Main d'œuvre directe</t>
+          <t>Gaz naturel</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>CC-PROD-003</t>
+          <t>CC-ENER-001</t>
         </is>
       </c>
     </row>
@@ -1470,17 +1470,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CC-PROD-003-PD2</t>
+          <t>CC-ENER-001-PD2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Consommables conditionnement</t>
+          <t>Électricité</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>CC-PROD-003</t>
+          <t>CC-ENER-001</t>
         </is>
       </c>
     </row>
@@ -1492,17 +1492,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CC-PROD-004-PD1</t>
+          <t>CC-LOG-002-PD1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Main d'œuvre directe</t>
+          <t>Transport routier</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>CC-PROD-004</t>
+          <t>CC-LOG-002</t>
         </is>
       </c>
     </row>
@@ -1514,17 +1514,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CC-PROD-004-PD2</t>
+          <t>CC-LOG-002-PD2</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Consommables conditionnement</t>
+          <t>Entreposage</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>CC-PROD-004</t>
+          <t>CC-LOG-002</t>
         </is>
       </c>
     </row>
@@ -1536,17 +1536,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CC-MAINT-001-PD1</t>
+          <t>CC-SGA-001-PD1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Pièces détachées</t>
+          <t>Publicité &amp; Media</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>CC-MAINT-001</t>
+          <t>CC-SGA-001</t>
         </is>
       </c>
     </row>
@@ -1558,17 +1558,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CC-MAINT-001-PD2</t>
+          <t>CC-SGA-001-PD2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Contrats de maintenance</t>
+          <t>Études de marché</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>CC-MAINT-001</t>
+          <t>CC-SGA-001</t>
         </is>
       </c>
     </row>
@@ -1580,17 +1580,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CC-ENER-001-PD1</t>
+          <t>CC-SGA-002-PD1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Gaz naturel</t>
+          <t>Commissions commerciales</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>CC-ENER-001</t>
+          <t>CC-SGA-002</t>
         </is>
       </c>
     </row>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CC-ENER-001-PD2</t>
+          <t>CC-SGA-002-PD2</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Électricité</t>
+          <t>Déplacements commerciaux</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>CC-ENER-001</t>
+          <t>CC-SGA-002</t>
         </is>
       </c>
     </row>
@@ -1624,17 +1624,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CC-LOG-002-PD1</t>
+          <t>CC-GA-001-PD1</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Transport routier</t>
+          <t>Licences logicielles</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>CC-LOG-002</t>
+          <t>CC-GA-001</t>
         </is>
       </c>
     </row>
@@ -1646,17 +1646,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CC-LOG-002-PD2</t>
+          <t>CC-GA-001-PD2</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Entreposage</t>
+          <t>Infrastructure Cloud</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>CC-LOG-002</t>
+          <t>CC-GA-001</t>
         </is>
       </c>
     </row>
@@ -1668,17 +1668,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CC-SGA-001-PD1</t>
+          <t>CC-GA-002-PD1</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Publicité &amp; Media</t>
+          <t>Formation</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>CC-SGA-001</t>
+          <t>CC-GA-002</t>
         </is>
       </c>
     </row>
@@ -1690,17 +1690,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>CC-SGA-001-PD2</t>
+          <t>CC-GA-002-PD2</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Études de marché</t>
+          <t>Recrutement</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>CC-SGA-001</t>
+          <t>CC-GA-002</t>
         </is>
       </c>
     </row>
@@ -1712,17 +1712,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>CC-SGA-002-PD1</t>
+          <t>CC-QUAL-001-PD1</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Commissions commerciales</t>
+          <t>Contrôles &amp; Analyses laboratoire</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>CC-SGA-002</t>
+          <t>CC-QUAL-001</t>
         </is>
       </c>
     </row>
@@ -1734,147 +1734,15 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CC-SGA-002-PD2</t>
+          <t>CC-QUAL-001-PD2</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Déplacements commerciaux</t>
+          <t>Certifications</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
-        <is>
-          <t>CC-SGA-002</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>CC-GA-001-PD1</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Licences logicielles</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>CC-GA-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>CC-GA-001-PD2</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Infrastructure Cloud</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>CC-GA-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>CC-GA-002-PD1</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Formation</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>CC-GA-002</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>CC-GA-002-PD2</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Recrutement</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>CC-GA-002</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>CC-QUAL-001-PD1</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Contrôles &amp; Analyses laboratoire</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>CC-QUAL-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>CC-QUAL-001-PD2</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Certifications</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
         <is>
           <t>CC-QUAL-001</t>
         </is>

</xml_diff>

<commit_message>
fix(demo): supprime les Centre de coût dupliqués dans l'arborescence financière (#53)
Les 6 lignes "Centre de coût" d'origine pointaient encore directement vers
le P&L (niveau grand-parent) au lieu de la nouvelle Catégorie intermédiaire,
et faisaient doublon avec les lignes équivalentes ajoutées pour le passage
à 4 étages. Cela provoquait une erreur d'import ("Code parent introuvable
dans le niveau Catégorie").

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/arborescence_financiere_demo.xlsx
+++ b/demo/arborescence_financiere_demo.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D66"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,132 +541,132 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CC-PROC-001</t>
+          <t>CAT-REV-PROD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Achats directs</t>
+          <t>Ventes Produits</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>REV</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CC-OPS-001</t>
+          <t>CAT-REV-SERV</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Prestations &amp; Services</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>REV</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CC-SGA-001</t>
+          <t>CAT-COGS-ACH</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Achats &amp; Approvisionnement</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SGA</t>
+          <t>COGS</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CC-SGA-002</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ventes</t>
+          <t>Production &amp; Industriel</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SGA</t>
+          <t>COGS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CC-GA-001</t>
+          <t>CAT-COGS-LOG</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Supply Chain &amp; Logistique</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>COGS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CC-GA-002</t>
+          <t>CAT-SGA-MKT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>SGA</t>
         </is>
       </c>
     </row>
@@ -678,17 +678,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAT-REV-PROD</t>
+          <t>CAT-SGA-VTE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ventes Produits</t>
+          <t>Ventes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>REV</t>
+          <t>SGA</t>
         </is>
       </c>
     </row>
@@ -700,17 +700,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CAT-REV-SERV</t>
+          <t>CAT-GA-SUP</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Prestations &amp; Services</t>
+          <t>Fonctions support</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>REV</t>
+          <t>GA</t>
         </is>
       </c>
     </row>
@@ -722,17 +722,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CAT-COGS-ACH</t>
+          <t>CAT-GA-IT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Achats &amp; Approvisionnement</t>
+          <t>IT &amp; Digital</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>GA</t>
         </is>
       </c>
     </row>
@@ -744,149 +744,149 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-GA-QUAL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Production &amp; Industriel</t>
+          <t>Qualité &amp; Conformité</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>GA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CAT-COGS-LOG</t>
+          <t>CC-PROC-001</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Supply Chain &amp; Logistique</t>
+          <t>Achats directs</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>CAT-COGS-ACH</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CAT-SGA-MKT</t>
+          <t>CC-PROC-002</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Achats indirects &amp; emballages</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SGA</t>
+          <t>CAT-COGS-ACH</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CAT-SGA-VTE</t>
+          <t>CC-OPS-001</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ventes</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>SGA</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CAT-GA-SUP</t>
+          <t>CC-PROD-001</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fonctions support</t>
+          <t>Production – Usine de Vitré</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAT-GA-IT</t>
+          <t>CC-PROD-002</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>IT &amp; Digital</t>
+          <t>Production – Usine de Hambourg</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Centre de coût</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAT-GA-QUAL</t>
+          <t>CC-PROD-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Qualité &amp; Conformité</t>
+          <t>Production – Usine de Valence</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
@@ -898,17 +898,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CC-PROC-001</t>
+          <t>CC-PROD-004</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Achats directs</t>
+          <t>Production – Usine de Green Bay</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CAT-COGS-ACH</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CC-PROC-002</t>
+          <t>CC-MAINT-001</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Achats indirects &amp; emballages</t>
+          <t>Maintenance industrielle</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CAT-COGS-ACH</t>
+          <t>CAT-COGS-PROD</t>
         </is>
       </c>
     </row>
@@ -942,12 +942,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CC-OPS-001</t>
+          <t>CC-ENER-001</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Énergie &amp; Utilités</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -964,17 +964,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CC-PROD-001</t>
+          <t>CC-LOG-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Production – Usine de Vitré</t>
+          <t>Logistique inter-usines</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-COGS-LOG</t>
         </is>
       </c>
     </row>
@@ -986,17 +986,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CC-PROD-002</t>
+          <t>CC-SGA-001</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Production – Usine de Hambourg</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-SGA-MKT</t>
         </is>
       </c>
     </row>
@@ -1008,17 +1008,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CC-PROD-003</t>
+          <t>CC-SGA-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Production – Usine de Valence</t>
+          <t>Ventes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-SGA-VTE</t>
         </is>
       </c>
     </row>
@@ -1030,17 +1030,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CC-PROD-004</t>
+          <t>CC-GA-001</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Production – Usine de Green Bay</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-GA-IT</t>
         </is>
       </c>
     </row>
@@ -1052,17 +1052,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CC-MAINT-001</t>
+          <t>CC-GA-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Maintenance industrielle</t>
+          <t>RH</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-GA-SUP</t>
         </is>
       </c>
     </row>
@@ -1074,149 +1074,149 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CC-ENER-001</t>
+          <t>CC-QUAL-001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Énergie &amp; Utilités</t>
+          <t>Qualité</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CAT-COGS-PROD</t>
+          <t>CAT-GA-QUAL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CC-LOG-002</t>
+          <t>CC-PROC-001-PD1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Logistique inter-usines</t>
+          <t>Matières premières</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CAT-COGS-LOG</t>
+          <t>CC-PROC-001</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CC-SGA-001</t>
+          <t>CC-PROC-001-PD2</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Emballages</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>CAT-SGA-MKT</t>
+          <t>CC-PROC-001</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CC-SGA-002</t>
+          <t>CC-PROC-002-PD1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ventes</t>
+          <t>Emballages plastiques</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CAT-SGA-VTE</t>
+          <t>CC-PROC-002</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CC-GA-001</t>
+          <t>CC-PROC-002-PD2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Fournitures indirectes</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CAT-GA-IT</t>
+          <t>CC-PROC-002</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CC-GA-002</t>
+          <t>CC-OPS-001-PD1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>Main d'œuvre directe</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>CAT-GA-SUP</t>
+          <t>CC-OPS-001</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Centre de coût</t>
+          <t>Poste de dépense</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CC-QUAL-001</t>
+          <t>CC-OPS-001-PD2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Qualité</t>
+          <t>Consommables production</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CAT-GA-QUAL</t>
+          <t>CC-OPS-001</t>
         </is>
       </c>
     </row>
@@ -1228,17 +1228,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CC-PROC-001-PD1</t>
+          <t>CC-PROD-001-PD1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Matières premières</t>
+          <t>Main d'œuvre directe</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CC-PROC-001</t>
+          <t>CC-PROD-001</t>
         </is>
       </c>
     </row>
@@ -1250,17 +1250,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CC-PROC-001-PD2</t>
+          <t>CC-PROD-001-PD2</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Emballages</t>
+          <t>Énergie ligne UHT</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CC-PROC-001</t>
+          <t>CC-PROD-001</t>
         </is>
       </c>
     </row>
@@ -1272,17 +1272,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CC-PROC-002-PD1</t>
+          <t>CC-PROD-002-PD1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Emballages plastiques</t>
+          <t>Main d'œuvre directe</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>CC-PROC-002</t>
+          <t>CC-PROD-002</t>
         </is>
       </c>
     </row>
@@ -1294,17 +1294,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CC-PROC-002-PD2</t>
+          <t>CC-PROD-002-PD2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Fournitures indirectes</t>
+          <t>Matière première laitière</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CC-PROC-002</t>
+          <t>CC-PROD-002</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CC-OPS-001-PD1</t>
+          <t>CC-PROD-003-PD1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CC-OPS-001</t>
+          <t>CC-PROD-003</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CC-OPS-001-PD2</t>
+          <t>CC-PROD-003-PD2</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Consommables production</t>
+          <t>Consommables conditionnement</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>CC-OPS-001</t>
+          <t>CC-PROD-003</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CC-PROD-001-PD1</t>
+          <t>CC-PROD-004-PD1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>CC-PROD-001</t>
+          <t>CC-PROD-004</t>
         </is>
       </c>
     </row>
@@ -1382,17 +1382,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CC-PROD-001-PD2</t>
+          <t>CC-PROD-004-PD2</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Énergie ligne UHT</t>
+          <t>Consommables conditionnement</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>CC-PROD-001</t>
+          <t>CC-PROD-004</t>
         </is>
       </c>
     </row>
@@ -1404,17 +1404,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CC-PROD-002-PD1</t>
+          <t>CC-MAINT-001-PD1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Main d'œuvre directe</t>
+          <t>Pièces détachées</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>CC-PROD-002</t>
+          <t>CC-MAINT-001</t>
         </is>
       </c>
     </row>
@@ -1426,17 +1426,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CC-PROD-002-PD2</t>
+          <t>CC-MAINT-001-PD2</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Matière première laitière</t>
+          <t>Contrats de maintenance</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>CC-PROD-002</t>
+          <t>CC-MAINT-001</t>
         </is>
       </c>
     </row>
@@ -1448,17 +1448,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CC-PROD-003-PD1</t>
+          <t>CC-ENER-001-PD1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Main d'œuvre directe</t>
+          <t>Gaz naturel</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>CC-PROD-003</t>
+          <t>CC-ENER-001</t>
         </is>
       </c>
     </row>
@@ -1470,17 +1470,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CC-PROD-003-PD2</t>
+          <t>CC-ENER-001-PD2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Consommables conditionnement</t>
+          <t>Électricité</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>CC-PROD-003</t>
+          <t>CC-ENER-001</t>
         </is>
       </c>
     </row>
@@ -1492,17 +1492,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CC-PROD-004-PD1</t>
+          <t>CC-LOG-002-PD1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Main d'œuvre directe</t>
+          <t>Transport routier</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>CC-PROD-004</t>
+          <t>CC-LOG-002</t>
         </is>
       </c>
     </row>
@@ -1514,17 +1514,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CC-PROD-004-PD2</t>
+          <t>CC-LOG-002-PD2</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Consommables conditionnement</t>
+          <t>Entreposage</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>CC-PROD-004</t>
+          <t>CC-LOG-002</t>
         </is>
       </c>
     </row>
@@ -1536,17 +1536,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CC-MAINT-001-PD1</t>
+          <t>CC-SGA-001-PD1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Pièces détachées</t>
+          <t>Publicité &amp; Media</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>CC-MAINT-001</t>
+          <t>CC-SGA-001</t>
         </is>
       </c>
     </row>
@@ -1558,17 +1558,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CC-MAINT-001-PD2</t>
+          <t>CC-SGA-001-PD2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Contrats de maintenance</t>
+          <t>Études de marché</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>CC-MAINT-001</t>
+          <t>CC-SGA-001</t>
         </is>
       </c>
     </row>
@@ -1580,17 +1580,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CC-ENER-001-PD1</t>
+          <t>CC-SGA-002-PD1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Gaz naturel</t>
+          <t>Commissions commerciales</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>CC-ENER-001</t>
+          <t>CC-SGA-002</t>
         </is>
       </c>
     </row>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CC-ENER-001-PD2</t>
+          <t>CC-SGA-002-PD2</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Électricité</t>
+          <t>Déplacements commerciaux</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>CC-ENER-001</t>
+          <t>CC-SGA-002</t>
         </is>
       </c>
     </row>
@@ -1624,17 +1624,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CC-LOG-002-PD1</t>
+          <t>CC-GA-001-PD1</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Transport routier</t>
+          <t>Licences logicielles</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>CC-LOG-002</t>
+          <t>CC-GA-001</t>
         </is>
       </c>
     </row>
@@ -1646,17 +1646,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CC-LOG-002-PD2</t>
+          <t>CC-GA-001-PD2</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Entreposage</t>
+          <t>Infrastructure Cloud</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>CC-LOG-002</t>
+          <t>CC-GA-001</t>
         </is>
       </c>
     </row>
@@ -1668,17 +1668,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CC-SGA-001-PD1</t>
+          <t>CC-GA-002-PD1</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Publicité &amp; Media</t>
+          <t>Formation</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>CC-SGA-001</t>
+          <t>CC-GA-002</t>
         </is>
       </c>
     </row>
@@ -1690,17 +1690,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>CC-SGA-001-PD2</t>
+          <t>CC-GA-002-PD2</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Études de marché</t>
+          <t>Recrutement</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>CC-SGA-001</t>
+          <t>CC-GA-002</t>
         </is>
       </c>
     </row>
@@ -1712,17 +1712,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>CC-SGA-002-PD1</t>
+          <t>CC-QUAL-001-PD1</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Commissions commerciales</t>
+          <t>Contrôles &amp; Analyses laboratoire</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>CC-SGA-002</t>
+          <t>CC-QUAL-001</t>
         </is>
       </c>
     </row>
@@ -1734,147 +1734,15 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CC-SGA-002-PD2</t>
+          <t>CC-QUAL-001-PD2</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Déplacements commerciaux</t>
+          <t>Certifications</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
-        <is>
-          <t>CC-SGA-002</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>CC-GA-001-PD1</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Licences logicielles</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>CC-GA-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>CC-GA-001-PD2</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Infrastructure Cloud</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>CC-GA-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>CC-GA-002-PD1</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Formation</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>CC-GA-002</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>CC-GA-002-PD2</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Recrutement</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>CC-GA-002</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>CC-QUAL-001-PD1</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Contrôles &amp; Analyses laboratoire</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>CC-QUAL-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Poste de dépense</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>CC-QUAL-001-PD2</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Certifications</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
         <is>
           <t>CC-QUAL-001</t>
         </is>

</xml_diff>